<commit_message>
feat: add ROS 2 collaboration skeleton
Add shared interfaces, heartbeat contracts, initialization skeleton,
launch profiles, hardware start blocking, static CI, and collaboration docs.
</commit_message>
<xml_diff>
--- a/구현_전_상세설계/01_노드_간_명령_이벤트_목록_초안.xlsx
+++ b/구현_전_상세설계/01_노드_간_명령_이벤트_목록_초안.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="사용 안내" sheetId="1" r:id="Rc96eee8732f54c9a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ROS 2 적용 기준" sheetId="2" r:id="Rcc14d3914711457d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="검토 질문" sheetId="3" r:id="Rad84a157b672452b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="통합 메시지 목록" sheetId="4" r:id="R5b4ec100608a4697"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="공통 Payload 정의" sheetId="5" r:id="R12e1844a803a4cd0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="전송·멱등 정책" sheetId="6" r:id="R3b4f65731ff7416c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="오류 코드 초안" sheetId="7" r:id="Rcf14abd6880149ea"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="사용 안내" sheetId="1" r:id="Rac9a1452813148de"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ROS 2 적용 기준" sheetId="2" r:id="Ra2ef82a43a56440b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="검토 질문" sheetId="3" r:id="R5b4809ac13654881"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="통합 메시지 목록" sheetId="4" r:id="R27f40a8b29124569"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="공통 Payload 정의" sheetId="5" r:id="R11d7891721074c9d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="전송·멱등 정책" sheetId="6" r:id="Rd8e612b5d44b4d7f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="오류 코드 초안" sheetId="7" r:id="R2e7fbea37162439e"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1195,15 +1195,11 @@
           <x:t xml:space="preserve">메시지 중요도별 별도 설정</x:t>
         </x:is>
       </x:c>
-      <x:c r="C13" s="35" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">SENSOR_DETECTED·물리 완료 이벤트는 Reliable, heartbeat는 Best Effort/Keep Last 1 검토</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D13" s="35" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">TODO(PARAM_TUNING)</x:t>
-        </x:is>
+      <x:c r="C13" s="35" t="str">
+        <x:v>SENSOR_DETECTED·물리 완료 이벤트는 Reliable, heartbeat는 Best Effort / Keep Last 1</x:v>
+      </x:c>
+      <x:c r="D13" s="35" t="str">
+        <x:v>확정 · POL-07 latest-only 정책에 따라 과거 샘플을 큐에 쌓지 않음</x:v>
       </x:c>
       <x:c r="E13" s="27"/>
       <x:c r="F13" s="27" t="n"/>

</xml_diff>